<commit_message>
Data analysis for PPE
Combined files to one dta
Created 8 figures by session or round
</commit_message>
<xml_diff>
--- a/cleaned_data/mgc9.xlsx
+++ b/cleaned_data/mgc9.xlsx
@@ -1,19 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ers725\Documents\Choice of Partners\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E816DD9-25D5-4620-8606-3E6B69FDE50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="833" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="20">
   <si>
     <t>session</t>
   </si>
@@ -78,7 +85,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -101,27 +108,338 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q409"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -174,7 +492,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:17">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -227,7 +545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:17">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -280,7 +598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:17">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -333,7 +651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:17">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -386,7 +704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:17">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -439,7 +757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:17">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -492,7 +810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:17">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -545,7 +863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:17">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -598,7 +916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:17">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -651,7 +969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:17">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -704,7 +1022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:17">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -757,7 +1075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:17">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -810,7 +1128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:17">
       <c r="A14" t="s">
         <v>1</v>
       </c>
@@ -863,7 +1181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:17">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -916,7 +1234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:17">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -969,7 +1287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:17">
       <c r="A17" t="s">
         <v>1</v>
       </c>
@@ -1022,7 +1340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:17">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -1075,7 +1393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:17">
       <c r="A19" t="s">
         <v>1</v>
       </c>
@@ -1128,7 +1446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:17">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -1181,7 +1499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:17">
       <c r="A21" t="s">
         <v>1</v>
       </c>
@@ -1234,7 +1552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:17">
       <c r="A22" t="s">
         <v>1</v>
       </c>
@@ -1287,7 +1605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:17">
       <c r="A23" t="s">
         <v>1</v>
       </c>
@@ -1340,7 +1658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:17">
       <c r="A24" t="s">
         <v>1</v>
       </c>
@@ -1393,7 +1711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:17">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -1446,7 +1764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:17">
       <c r="A26" t="s">
         <v>1</v>
       </c>
@@ -1499,7 +1817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:17">
       <c r="A27" t="s">
         <v>1</v>
       </c>
@@ -1528,10 +1846,10 @@
         <v>1</v>
       </c>
       <c r="J27" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K27" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L27" s="1">
         <v>2</v>
@@ -1552,7 +1870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:17">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -1605,7 +1923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:17">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -1658,7 +1976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:17">
       <c r="A30" t="s">
         <v>1</v>
       </c>
@@ -1711,7 +2029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:17">
       <c r="A31" t="s">
         <v>1</v>
       </c>
@@ -1764,7 +2082,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:17">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -1817,7 +2135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:17">
       <c r="A33" t="s">
         <v>1</v>
       </c>
@@ -1870,7 +2188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:17">
       <c r="A34" t="s">
         <v>1</v>
       </c>
@@ -1923,7 +2241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:17">
       <c r="A35" t="s">
         <v>1</v>
       </c>
@@ -1976,7 +2294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:17">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -2029,7 +2347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:17">
       <c r="A37" t="s">
         <v>1</v>
       </c>
@@ -2082,7 +2400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:17">
       <c r="A38" t="s">
         <v>1</v>
       </c>
@@ -2135,7 +2453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:17">
       <c r="A39" t="s">
         <v>1</v>
       </c>
@@ -2188,7 +2506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:17">
       <c r="A40" t="s">
         <v>1</v>
       </c>
@@ -2241,7 +2559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:17">
       <c r="A41" t="s">
         <v>1</v>
       </c>
@@ -2294,7 +2612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:17">
       <c r="A42" t="s">
         <v>1</v>
       </c>
@@ -2347,7 +2665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:17">
       <c r="A43" t="s">
         <v>1</v>
       </c>
@@ -2400,7 +2718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:17">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -2453,7 +2771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:17">
       <c r="A45" t="s">
         <v>1</v>
       </c>
@@ -2506,7 +2824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:17">
       <c r="A46" t="s">
         <v>1</v>
       </c>
@@ -2559,7 +2877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:17">
       <c r="A47" t="s">
         <v>1</v>
       </c>
@@ -2612,7 +2930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:17">
       <c r="A48" t="s">
         <v>1</v>
       </c>
@@ -2665,7 +2983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:17">
       <c r="A49" t="s">
         <v>1</v>
       </c>
@@ -2718,7 +3036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:17">
       <c r="A50" t="s">
         <v>1</v>
       </c>
@@ -2771,7 +3089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:17">
       <c r="A51" t="s">
         <v>1</v>
       </c>
@@ -2824,7 +3142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:17">
       <c r="A52" t="s">
         <v>1</v>
       </c>
@@ -2877,7 +3195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:17">
       <c r="A53" t="s">
         <v>1</v>
       </c>
@@ -2930,7 +3248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:17">
       <c r="A54" t="s">
         <v>1</v>
       </c>
@@ -2983,7 +3301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:17">
       <c r="A55" t="s">
         <v>1</v>
       </c>
@@ -3036,7 +3354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:17">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -3089,7 +3407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:17">
       <c r="A57" t="s">
         <v>1</v>
       </c>
@@ -3142,7 +3460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:17">
       <c r="A58" t="s">
         <v>1</v>
       </c>
@@ -3195,7 +3513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:17">
       <c r="A59" t="s">
         <v>1</v>
       </c>
@@ -3248,7 +3566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:17">
       <c r="A60" t="s">
         <v>1</v>
       </c>
@@ -3301,7 +3619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:17">
       <c r="A61" t="s">
         <v>1</v>
       </c>
@@ -3354,7 +3672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:17">
       <c r="A62" t="s">
         <v>1</v>
       </c>
@@ -3407,7 +3725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:17">
       <c r="A63" t="s">
         <v>1</v>
       </c>
@@ -3460,7 +3778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:17">
       <c r="A64" t="s">
         <v>1</v>
       </c>
@@ -3513,7 +3831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:17">
       <c r="A65" t="s">
         <v>1</v>
       </c>
@@ -3566,7 +3884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:17">
       <c r="A66" t="s">
         <v>1</v>
       </c>
@@ -3619,7 +3937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:17">
       <c r="A67" t="s">
         <v>1</v>
       </c>
@@ -3672,7 +3990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:17">
       <c r="A68" t="s">
         <v>1</v>
       </c>
@@ -3725,7 +4043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:17">
       <c r="A69" t="s">
         <v>1</v>
       </c>
@@ -3778,7 +4096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:17">
       <c r="A70" t="s">
         <v>1</v>
       </c>
@@ -3831,7 +4149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:17">
       <c r="A71" t="s">
         <v>1</v>
       </c>
@@ -3884,7 +4202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:17">
       <c r="A72" t="s">
         <v>1</v>
       </c>
@@ -3937,7 +4255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:17">
       <c r="A73" t="s">
         <v>1</v>
       </c>
@@ -3990,7 +4308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:17">
       <c r="A74" t="s">
         <v>1</v>
       </c>
@@ -4043,7 +4361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:17">
       <c r="A75" t="s">
         <v>1</v>
       </c>
@@ -4096,7 +4414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:17">
       <c r="A76" t="s">
         <v>1</v>
       </c>
@@ -4149,7 +4467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:17">
       <c r="A77" t="s">
         <v>1</v>
       </c>
@@ -4202,7 +4520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:17">
       <c r="A78" t="s">
         <v>1</v>
       </c>
@@ -4255,7 +4573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:17">
       <c r="A79" t="s">
         <v>1</v>
       </c>
@@ -4308,7 +4626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:17">
       <c r="A80" t="s">
         <v>1</v>
       </c>
@@ -4361,7 +4679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:17">
       <c r="A81" t="s">
         <v>1</v>
       </c>
@@ -4414,7 +4732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:17">
       <c r="A82" t="s">
         <v>1</v>
       </c>
@@ -4467,7 +4785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:17">
       <c r="A83" t="s">
         <v>1</v>
       </c>
@@ -4520,7 +4838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:17">
       <c r="A84" t="s">
         <v>1</v>
       </c>
@@ -4573,7 +4891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:17">
       <c r="A85" t="s">
         <v>1</v>
       </c>
@@ -4626,7 +4944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:17">
       <c r="A86" t="s">
         <v>1</v>
       </c>
@@ -4679,7 +4997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:17">
       <c r="A87" t="s">
         <v>1</v>
       </c>
@@ -4732,7 +5050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:17">
       <c r="A88" t="s">
         <v>1</v>
       </c>
@@ -4785,7 +5103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:17">
       <c r="A89" t="s">
         <v>1</v>
       </c>
@@ -4838,7 +5156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:17">
       <c r="A90" t="s">
         <v>1</v>
       </c>
@@ -4891,7 +5209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:17">
       <c r="A91" t="s">
         <v>1</v>
       </c>
@@ -4944,7 +5262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:17">
       <c r="A92" t="s">
         <v>1</v>
       </c>
@@ -4997,7 +5315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:17">
       <c r="A93" t="s">
         <v>1</v>
       </c>
@@ -5050,7 +5368,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:17">
       <c r="A94" t="s">
         <v>1</v>
       </c>
@@ -5103,7 +5421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:17">
       <c r="A95" t="s">
         <v>1</v>
       </c>
@@ -5156,7 +5474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:17">
       <c r="A96" t="s">
         <v>1</v>
       </c>
@@ -5209,7 +5527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:17">
       <c r="A97" t="s">
         <v>1</v>
       </c>
@@ -5262,7 +5580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:17">
       <c r="A98" t="s">
         <v>1</v>
       </c>
@@ -5315,7 +5633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:17">
       <c r="A99" t="s">
         <v>1</v>
       </c>
@@ -5368,7 +5686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:17">
       <c r="A100" t="s">
         <v>1</v>
       </c>
@@ -5421,7 +5739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:17">
       <c r="A101" t="s">
         <v>1</v>
       </c>
@@ -5474,7 +5792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:17">
       <c r="A102" t="s">
         <v>1</v>
       </c>
@@ -5527,7 +5845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:17">
       <c r="A103" t="s">
         <v>1</v>
       </c>
@@ -5580,7 +5898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:17">
       <c r="A104" t="s">
         <v>1</v>
       </c>
@@ -5633,7 +5951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:17">
       <c r="A105" t="s">
         <v>1</v>
       </c>
@@ -5686,7 +6004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:17">
       <c r="A106" t="s">
         <v>1</v>
       </c>
@@ -5739,7 +6057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:17">
       <c r="A107" t="s">
         <v>1</v>
       </c>
@@ -5792,7 +6110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:17">
       <c r="A108" t="s">
         <v>1</v>
       </c>
@@ -5845,7 +6163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:17">
       <c r="A109" t="s">
         <v>1</v>
       </c>
@@ -5898,7 +6216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:17">
       <c r="A110" t="s">
         <v>1</v>
       </c>
@@ -5951,7 +6269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:17">
       <c r="A111" t="s">
         <v>1</v>
       </c>
@@ -6004,7 +6322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:17">
       <c r="A112" t="s">
         <v>1</v>
       </c>
@@ -6057,7 +6375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:17">
       <c r="A113" t="s">
         <v>1</v>
       </c>
@@ -6110,7 +6428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:17">
       <c r="A114" t="s">
         <v>1</v>
       </c>
@@ -6163,7 +6481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:17">
       <c r="A115" t="s">
         <v>1</v>
       </c>
@@ -6216,7 +6534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:17">
       <c r="A116" t="s">
         <v>1</v>
       </c>
@@ -6269,7 +6587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" spans="1:17">
       <c r="A117" t="s">
         <v>1</v>
       </c>
@@ -6322,7 +6640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:17">
       <c r="A118" t="s">
         <v>1</v>
       </c>
@@ -6375,7 +6693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:17">
       <c r="A119" t="s">
         <v>1</v>
       </c>
@@ -6428,7 +6746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:17">
       <c r="A120" t="s">
         <v>1</v>
       </c>
@@ -6481,7 +6799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:17">
       <c r="A121" t="s">
         <v>1</v>
       </c>
@@ -6534,7 +6852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" spans="1:17">
       <c r="A122" t="s">
         <v>1</v>
       </c>
@@ -6587,7 +6905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:17">
       <c r="A123" t="s">
         <v>1</v>
       </c>
@@ -6640,7 +6958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" spans="1:17">
       <c r="A124" t="s">
         <v>1</v>
       </c>
@@ -6693,7 +7011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" spans="1:17">
       <c r="A125" t="s">
         <v>1</v>
       </c>
@@ -6746,7 +7064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" spans="1:17">
       <c r="A126" t="s">
         <v>1</v>
       </c>
@@ -6799,7 +7117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" spans="1:17">
       <c r="A127" t="s">
         <v>1</v>
       </c>
@@ -6852,7 +7170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" spans="1:17">
       <c r="A128" t="s">
         <v>1</v>
       </c>
@@ -6905,7 +7223,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" spans="1:17">
       <c r="A129" t="s">
         <v>1</v>
       </c>
@@ -6958,7 +7276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" spans="1:17">
       <c r="A130" t="s">
         <v>1</v>
       </c>
@@ -7011,7 +7329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" spans="1:17">
       <c r="A131" t="s">
         <v>1</v>
       </c>
@@ -7064,7 +7382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" spans="1:17">
       <c r="A132" t="s">
         <v>1</v>
       </c>
@@ -7117,7 +7435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" spans="1:17">
       <c r="A133" t="s">
         <v>1</v>
       </c>
@@ -7170,7 +7488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" spans="1:17">
       <c r="A134" t="s">
         <v>1</v>
       </c>
@@ -7223,7 +7541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" spans="1:17">
       <c r="A135" t="s">
         <v>1</v>
       </c>
@@ -7276,7 +7594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" spans="1:17">
       <c r="A136" t="s">
         <v>1</v>
       </c>
@@ -7329,7 +7647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" spans="1:17">
       <c r="A137" t="s">
         <v>1</v>
       </c>
@@ -7382,7 +7700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" spans="1:17">
       <c r="A138" t="s">
         <v>1</v>
       </c>
@@ -7435,7 +7753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139">
+    <row r="139" spans="1:17">
       <c r="A139" t="s">
         <v>1</v>
       </c>
@@ -7488,7 +7806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" spans="1:17">
       <c r="A140" t="s">
         <v>1</v>
       </c>
@@ -7541,7 +7859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" spans="1:17">
       <c r="A141" t="s">
         <v>1</v>
       </c>
@@ -7594,7 +7912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" spans="1:17">
       <c r="A142" t="s">
         <v>1</v>
       </c>
@@ -7647,7 +7965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" spans="1:17">
       <c r="A143" t="s">
         <v>1</v>
       </c>
@@ -7700,7 +8018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" spans="1:17">
       <c r="A144" t="s">
         <v>1</v>
       </c>
@@ -7753,7 +8071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" spans="1:17">
       <c r="A145" t="s">
         <v>1</v>
       </c>
@@ -7806,7 +8124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" spans="1:17">
       <c r="A146" t="s">
         <v>1</v>
       </c>
@@ -7859,7 +8177,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" spans="1:17">
       <c r="A147" t="s">
         <v>1</v>
       </c>
@@ -7912,7 +8230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" spans="1:17">
       <c r="A148" t="s">
         <v>1</v>
       </c>
@@ -7965,7 +8283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" spans="1:17">
       <c r="A149" t="s">
         <v>1</v>
       </c>
@@ -8018,7 +8336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" spans="1:17">
       <c r="A150" t="s">
         <v>1</v>
       </c>
@@ -8071,7 +8389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" spans="1:17">
       <c r="A151" t="s">
         <v>1</v>
       </c>
@@ -8124,7 +8442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" spans="1:17">
       <c r="A152" t="s">
         <v>1</v>
       </c>
@@ -8177,7 +8495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153">
+    <row r="153" spans="1:17">
       <c r="A153" t="s">
         <v>1</v>
       </c>
@@ -8230,7 +8548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154">
+    <row r="154" spans="1:17">
       <c r="A154" t="s">
         <v>1</v>
       </c>
@@ -8283,7 +8601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155">
+    <row r="155" spans="1:17">
       <c r="A155" t="s">
         <v>1</v>
       </c>
@@ -8336,7 +8654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156">
+    <row r="156" spans="1:17">
       <c r="A156" t="s">
         <v>1</v>
       </c>
@@ -8389,7 +8707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157">
+    <row r="157" spans="1:17">
       <c r="A157" t="s">
         <v>1</v>
       </c>
@@ -8442,7 +8760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158">
+    <row r="158" spans="1:17">
       <c r="A158" t="s">
         <v>1</v>
       </c>
@@ -8495,7 +8813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" spans="1:17">
       <c r="A159" t="s">
         <v>1</v>
       </c>
@@ -8548,7 +8866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" spans="1:17">
       <c r="A160" t="s">
         <v>1</v>
       </c>
@@ -8601,7 +8919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" spans="1:17">
       <c r="A161" t="s">
         <v>1</v>
       </c>
@@ -8654,7 +8972,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162">
+    <row r="162" spans="1:17">
       <c r="A162" t="s">
         <v>1</v>
       </c>
@@ -8707,7 +9025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163">
+    <row r="163" spans="1:17">
       <c r="A163" t="s">
         <v>1</v>
       </c>
@@ -8760,7 +9078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" spans="1:17">
       <c r="A164" t="s">
         <v>1</v>
       </c>
@@ -8813,7 +9131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165">
+    <row r="165" spans="1:17">
       <c r="A165" t="s">
         <v>1</v>
       </c>
@@ -8866,7 +9184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166">
+    <row r="166" spans="1:17">
       <c r="A166" t="s">
         <v>1</v>
       </c>
@@ -8919,7 +9237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167">
+    <row r="167" spans="1:17">
       <c r="A167" t="s">
         <v>1</v>
       </c>
@@ -8972,7 +9290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168">
+    <row r="168" spans="1:17">
       <c r="A168" t="s">
         <v>1</v>
       </c>
@@ -9025,7 +9343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169">
+    <row r="169" spans="1:17">
       <c r="A169" t="s">
         <v>1</v>
       </c>
@@ -9078,7 +9396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170">
+    <row r="170" spans="1:17">
       <c r="A170" t="s">
         <v>1</v>
       </c>
@@ -9131,7 +9449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171">
+    <row r="171" spans="1:17">
       <c r="A171" t="s">
         <v>1</v>
       </c>
@@ -9184,7 +9502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172">
+    <row r="172" spans="1:17">
       <c r="A172" t="s">
         <v>1</v>
       </c>
@@ -9237,7 +9555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173">
+    <row r="173" spans="1:17">
       <c r="A173" t="s">
         <v>1</v>
       </c>
@@ -9290,7 +9608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174">
+    <row r="174" spans="1:17">
       <c r="A174" t="s">
         <v>1</v>
       </c>
@@ -9343,7 +9661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175">
+    <row r="175" spans="1:17">
       <c r="A175" t="s">
         <v>1</v>
       </c>
@@ -9396,7 +9714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176">
+    <row r="176" spans="1:17">
       <c r="A176" t="s">
         <v>1</v>
       </c>
@@ -9449,7 +9767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177">
+    <row r="177" spans="1:17">
       <c r="A177" t="s">
         <v>1</v>
       </c>
@@ -9502,7 +9820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178">
+    <row r="178" spans="1:17">
       <c r="A178" t="s">
         <v>1</v>
       </c>
@@ -9555,7 +9873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179">
+    <row r="179" spans="1:17">
       <c r="A179" t="s">
         <v>1</v>
       </c>
@@ -9608,7 +9926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180">
+    <row r="180" spans="1:17">
       <c r="A180" t="s">
         <v>1</v>
       </c>
@@ -9661,7 +9979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181">
+    <row r="181" spans="1:17">
       <c r="A181" t="s">
         <v>1</v>
       </c>
@@ -9714,7 +10032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182">
+    <row r="182" spans="1:17">
       <c r="A182" t="s">
         <v>1</v>
       </c>
@@ -9767,7 +10085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183">
+    <row r="183" spans="1:17">
       <c r="A183" t="s">
         <v>1</v>
       </c>
@@ -9820,7 +10138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184">
+    <row r="184" spans="1:17">
       <c r="A184" t="s">
         <v>1</v>
       </c>
@@ -9873,7 +10191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185">
+    <row r="185" spans="1:17">
       <c r="A185" t="s">
         <v>1</v>
       </c>
@@ -9926,7 +10244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186">
+    <row r="186" spans="1:17">
       <c r="A186" t="s">
         <v>1</v>
       </c>
@@ -9979,7 +10297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187">
+    <row r="187" spans="1:17">
       <c r="A187" t="s">
         <v>1</v>
       </c>
@@ -10032,7 +10350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188">
+    <row r="188" spans="1:17">
       <c r="A188" t="s">
         <v>1</v>
       </c>
@@ -10085,7 +10403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189">
+    <row r="189" spans="1:17">
       <c r="A189" t="s">
         <v>1</v>
       </c>
@@ -10138,7 +10456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190">
+    <row r="190" spans="1:17">
       <c r="A190" t="s">
         <v>1</v>
       </c>
@@ -10191,7 +10509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191">
+    <row r="191" spans="1:17">
       <c r="A191" t="s">
         <v>1</v>
       </c>
@@ -10244,7 +10562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192">
+    <row r="192" spans="1:17">
       <c r="A192" t="s">
         <v>1</v>
       </c>
@@ -10297,7 +10615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193">
+    <row r="193" spans="1:17">
       <c r="A193" t="s">
         <v>1</v>
       </c>
@@ -10350,7 +10668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194">
+    <row r="194" spans="1:17">
       <c r="A194" t="s">
         <v>1</v>
       </c>
@@ -10403,7 +10721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195">
+    <row r="195" spans="1:17">
       <c r="A195" t="s">
         <v>1</v>
       </c>
@@ -10456,7 +10774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196">
+    <row r="196" spans="1:17">
       <c r="A196" t="s">
         <v>1</v>
       </c>
@@ -10509,7 +10827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197">
+    <row r="197" spans="1:17">
       <c r="A197" t="s">
         <v>1</v>
       </c>
@@ -10562,7 +10880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198">
+    <row r="198" spans="1:17">
       <c r="A198" t="s">
         <v>1</v>
       </c>
@@ -10615,7 +10933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199">
+    <row r="199" spans="1:17">
       <c r="A199" t="s">
         <v>1</v>
       </c>
@@ -10668,7 +10986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200">
+    <row r="200" spans="1:17">
       <c r="A200" t="s">
         <v>1</v>
       </c>
@@ -10721,7 +11039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201">
+    <row r="201" spans="1:17">
       <c r="A201" t="s">
         <v>1</v>
       </c>
@@ -10774,7 +11092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202">
+    <row r="202" spans="1:17">
       <c r="A202" t="s">
         <v>1</v>
       </c>
@@ -10827,7 +11145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203">
+    <row r="203" spans="1:17">
       <c r="A203" t="s">
         <v>1</v>
       </c>
@@ -10880,7 +11198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204">
+    <row r="204" spans="1:17">
       <c r="A204" t="s">
         <v>1</v>
       </c>
@@ -10933,7 +11251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205">
+    <row r="205" spans="1:17">
       <c r="A205" t="s">
         <v>1</v>
       </c>
@@ -10986,7 +11304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206">
+    <row r="206" spans="1:17">
       <c r="A206" t="s">
         <v>1</v>
       </c>
@@ -11039,7 +11357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207">
+    <row r="207" spans="1:17">
       <c r="A207" t="s">
         <v>1</v>
       </c>
@@ -11092,7 +11410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208">
+    <row r="208" spans="1:17">
       <c r="A208" t="s">
         <v>1</v>
       </c>
@@ -11145,7 +11463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209">
+    <row r="209" spans="1:17">
       <c r="A209" t="s">
         <v>1</v>
       </c>
@@ -11198,7 +11516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210">
+    <row r="210" spans="1:17">
       <c r="A210" t="s">
         <v>1</v>
       </c>
@@ -11251,7 +11569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211">
+    <row r="211" spans="1:17">
       <c r="A211" t="s">
         <v>1</v>
       </c>
@@ -11304,7 +11622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212">
+    <row r="212" spans="1:17">
       <c r="A212" t="s">
         <v>1</v>
       </c>
@@ -11357,7 +11675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213">
+    <row r="213" spans="1:17">
       <c r="A213" t="s">
         <v>1</v>
       </c>
@@ -11410,7 +11728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214">
+    <row r="214" spans="1:17">
       <c r="A214" t="s">
         <v>1</v>
       </c>
@@ -11463,7 +11781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215">
+    <row r="215" spans="1:17">
       <c r="A215" t="s">
         <v>1</v>
       </c>
@@ -11516,7 +11834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216">
+    <row r="216" spans="1:17">
       <c r="A216" t="s">
         <v>1</v>
       </c>
@@ -11569,7 +11887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217">
+    <row r="217" spans="1:17">
       <c r="A217" t="s">
         <v>1</v>
       </c>
@@ -11622,7 +11940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218">
+    <row r="218" spans="1:17">
       <c r="A218" t="s">
         <v>1</v>
       </c>
@@ -11675,7 +11993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219">
+    <row r="219" spans="1:17">
       <c r="A219" t="s">
         <v>1</v>
       </c>
@@ -11728,7 +12046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220">
+    <row r="220" spans="1:17">
       <c r="A220" t="s">
         <v>1</v>
       </c>
@@ -11781,7 +12099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221">
+    <row r="221" spans="1:17">
       <c r="A221" t="s">
         <v>1</v>
       </c>
@@ -11834,7 +12152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222">
+    <row r="222" spans="1:17">
       <c r="A222" t="s">
         <v>1</v>
       </c>
@@ -11887,7 +12205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223">
+    <row r="223" spans="1:17">
       <c r="A223" t="s">
         <v>1</v>
       </c>
@@ -11940,7 +12258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224">
+    <row r="224" spans="1:17">
       <c r="A224" t="s">
         <v>1</v>
       </c>
@@ -11993,7 +12311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225">
+    <row r="225" spans="1:17">
       <c r="A225" t="s">
         <v>1</v>
       </c>
@@ -12046,7 +12364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226">
+    <row r="226" spans="1:17">
       <c r="A226" t="s">
         <v>1</v>
       </c>
@@ -12099,7 +12417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227">
+    <row r="227" spans="1:17">
       <c r="A227" t="s">
         <v>1</v>
       </c>
@@ -12152,7 +12470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228">
+    <row r="228" spans="1:17">
       <c r="A228" t="s">
         <v>1</v>
       </c>
@@ -12205,7 +12523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229">
+    <row r="229" spans="1:17">
       <c r="A229" t="s">
         <v>1</v>
       </c>
@@ -12258,7 +12576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230">
+    <row r="230" spans="1:17">
       <c r="A230" t="s">
         <v>1</v>
       </c>
@@ -12311,7 +12629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231">
+    <row r="231" spans="1:17">
       <c r="A231" t="s">
         <v>1</v>
       </c>
@@ -12364,7 +12682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232">
+    <row r="232" spans="1:17">
       <c r="A232" t="s">
         <v>1</v>
       </c>
@@ -12417,7 +12735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233">
+    <row r="233" spans="1:17">
       <c r="A233" t="s">
         <v>1</v>
       </c>
@@ -12470,7 +12788,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234">
+    <row r="234" spans="1:17">
       <c r="A234" t="s">
         <v>1</v>
       </c>
@@ -12523,7 +12841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235">
+    <row r="235" spans="1:17">
       <c r="A235" t="s">
         <v>1</v>
       </c>
@@ -12576,7 +12894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236">
+    <row r="236" spans="1:17">
       <c r="A236" t="s">
         <v>1</v>
       </c>
@@ -12629,7 +12947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237">
+    <row r="237" spans="1:17">
       <c r="A237" t="s">
         <v>1</v>
       </c>
@@ -12682,7 +13000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238">
+    <row r="238" spans="1:17">
       <c r="A238" t="s">
         <v>1</v>
       </c>
@@ -12735,7 +13053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239">
+    <row r="239" spans="1:17">
       <c r="A239" t="s">
         <v>1</v>
       </c>
@@ -12788,7 +13106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240">
+    <row r="240" spans="1:17">
       <c r="A240" t="s">
         <v>1</v>
       </c>
@@ -12841,7 +13159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241">
+    <row r="241" spans="1:17">
       <c r="A241" t="s">
         <v>1</v>
       </c>
@@ -12894,7 +13212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242">
+    <row r="242" spans="1:17">
       <c r="A242" t="s">
         <v>1</v>
       </c>
@@ -12947,7 +13265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243">
+    <row r="243" spans="1:17">
       <c r="A243" t="s">
         <v>1</v>
       </c>
@@ -13000,7 +13318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244">
+    <row r="244" spans="1:17">
       <c r="A244" t="s">
         <v>1</v>
       </c>
@@ -13053,7 +13371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245">
+    <row r="245" spans="1:17">
       <c r="A245" t="s">
         <v>1</v>
       </c>
@@ -13106,7 +13424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246">
+    <row r="246" spans="1:17">
       <c r="A246" t="s">
         <v>1</v>
       </c>
@@ -13159,7 +13477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247">
+    <row r="247" spans="1:17">
       <c r="A247" t="s">
         <v>1</v>
       </c>
@@ -13212,7 +13530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248">
+    <row r="248" spans="1:17">
       <c r="A248" t="s">
         <v>1</v>
       </c>
@@ -13265,7 +13583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249">
+    <row r="249" spans="1:17">
       <c r="A249" t="s">
         <v>1</v>
       </c>
@@ -13318,7 +13636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="250">
+    <row r="250" spans="1:17">
       <c r="A250" t="s">
         <v>1</v>
       </c>
@@ -13371,7 +13689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251">
+    <row r="251" spans="1:17">
       <c r="A251" t="s">
         <v>1</v>
       </c>
@@ -13424,7 +13742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252">
+    <row r="252" spans="1:17">
       <c r="A252" t="s">
         <v>1</v>
       </c>
@@ -13477,7 +13795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253">
+    <row r="253" spans="1:17">
       <c r="A253" t="s">
         <v>1</v>
       </c>
@@ -13530,7 +13848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254">
+    <row r="254" spans="1:17">
       <c r="A254" t="s">
         <v>1</v>
       </c>
@@ -13583,7 +13901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255">
+    <row r="255" spans="1:17">
       <c r="A255" t="s">
         <v>1</v>
       </c>
@@ -13636,7 +13954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256">
+    <row r="256" spans="1:17">
       <c r="A256" t="s">
         <v>1</v>
       </c>
@@ -13689,7 +14007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="257">
+    <row r="257" spans="1:17">
       <c r="A257" t="s">
         <v>1</v>
       </c>
@@ -13742,7 +14060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="258">
+    <row r="258" spans="1:17">
       <c r="A258" t="s">
         <v>1</v>
       </c>
@@ -13795,7 +14113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259">
+    <row r="259" spans="1:17">
       <c r="A259" t="s">
         <v>1</v>
       </c>
@@ -13848,7 +14166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="260">
+    <row r="260" spans="1:17">
       <c r="A260" t="s">
         <v>1</v>
       </c>
@@ -13901,7 +14219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261">
+    <row r="261" spans="1:17">
       <c r="A261" t="s">
         <v>1</v>
       </c>
@@ -13954,7 +14272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="262">
+    <row r="262" spans="1:17">
       <c r="A262" t="s">
         <v>1</v>
       </c>
@@ -14007,7 +14325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="263">
+    <row r="263" spans="1:17">
       <c r="A263" t="s">
         <v>1</v>
       </c>
@@ -14060,7 +14378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="264">
+    <row r="264" spans="1:17">
       <c r="A264" t="s">
         <v>1</v>
       </c>
@@ -14113,7 +14431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265">
+    <row r="265" spans="1:17">
       <c r="A265" t="s">
         <v>1</v>
       </c>
@@ -14166,7 +14484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="266">
+    <row r="266" spans="1:17">
       <c r="A266" t="s">
         <v>1</v>
       </c>
@@ -14219,7 +14537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267">
+    <row r="267" spans="1:17">
       <c r="A267" t="s">
         <v>1</v>
       </c>
@@ -14272,7 +14590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268">
+    <row r="268" spans="1:17">
       <c r="A268" t="s">
         <v>1</v>
       </c>
@@ -14325,7 +14643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269">
+    <row r="269" spans="1:17">
       <c r="A269" t="s">
         <v>1</v>
       </c>
@@ -14378,7 +14696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270">
+    <row r="270" spans="1:17">
       <c r="A270" t="s">
         <v>1</v>
       </c>
@@ -14431,7 +14749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271">
+    <row r="271" spans="1:17">
       <c r="A271" t="s">
         <v>1</v>
       </c>
@@ -14484,7 +14802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="272">
+    <row r="272" spans="1:17">
       <c r="A272" t="s">
         <v>1</v>
       </c>
@@ -14537,7 +14855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="273">
+    <row r="273" spans="1:17">
       <c r="A273" t="s">
         <v>1</v>
       </c>
@@ -14590,7 +14908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="274">
+    <row r="274" spans="1:17">
       <c r="A274" t="s">
         <v>1</v>
       </c>
@@ -14643,7 +14961,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275">
+    <row r="275" spans="1:17">
       <c r="A275" t="s">
         <v>1</v>
       </c>
@@ -14696,7 +15014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276">
+    <row r="276" spans="1:17">
       <c r="A276" t="s">
         <v>1</v>
       </c>
@@ -14749,7 +15067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="277">
+    <row r="277" spans="1:17">
       <c r="A277" t="s">
         <v>1</v>
       </c>
@@ -14802,7 +15120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278">
+    <row r="278" spans="1:17">
       <c r="A278" t="s">
         <v>1</v>
       </c>
@@ -14855,7 +15173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279">
+    <row r="279" spans="1:17">
       <c r="A279" t="s">
         <v>1</v>
       </c>
@@ -14908,7 +15226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280">
+    <row r="280" spans="1:17">
       <c r="A280" t="s">
         <v>1</v>
       </c>
@@ -14961,7 +15279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281">
+    <row r="281" spans="1:17">
       <c r="A281" t="s">
         <v>1</v>
       </c>
@@ -15014,7 +15332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282">
+    <row r="282" spans="1:17">
       <c r="A282" t="s">
         <v>1</v>
       </c>
@@ -15067,7 +15385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283">
+    <row r="283" spans="1:17">
       <c r="A283" t="s">
         <v>1</v>
       </c>
@@ -15120,7 +15438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284">
+    <row r="284" spans="1:17">
       <c r="A284" t="s">
         <v>1</v>
       </c>
@@ -15173,7 +15491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285">
+    <row r="285" spans="1:17">
       <c r="A285" t="s">
         <v>1</v>
       </c>
@@ -15226,7 +15544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286">
+    <row r="286" spans="1:17">
       <c r="A286" t="s">
         <v>1</v>
       </c>
@@ -15279,7 +15597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287">
+    <row r="287" spans="1:17">
       <c r="A287" t="s">
         <v>1</v>
       </c>
@@ -15332,7 +15650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288">
+    <row r="288" spans="1:17">
       <c r="A288" t="s">
         <v>1</v>
       </c>
@@ -15385,7 +15703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="289">
+    <row r="289" spans="1:17">
       <c r="A289" t="s">
         <v>1</v>
       </c>
@@ -15438,7 +15756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="290">
+    <row r="290" spans="1:17">
       <c r="A290" t="s">
         <v>1</v>
       </c>
@@ -15491,7 +15809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="291">
+    <row r="291" spans="1:17">
       <c r="A291" t="s">
         <v>1</v>
       </c>
@@ -15544,7 +15862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="292">
+    <row r="292" spans="1:17">
       <c r="A292" t="s">
         <v>1</v>
       </c>
@@ -15597,7 +15915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="293">
+    <row r="293" spans="1:17">
       <c r="A293" t="s">
         <v>1</v>
       </c>
@@ -15650,7 +15968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294">
+    <row r="294" spans="1:17">
       <c r="A294" t="s">
         <v>1</v>
       </c>
@@ -15703,7 +16021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295">
+    <row r="295" spans="1:17">
       <c r="A295" t="s">
         <v>1</v>
       </c>
@@ -15756,7 +16074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296">
+    <row r="296" spans="1:17">
       <c r="A296" t="s">
         <v>1</v>
       </c>
@@ -15809,7 +16127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297">
+    <row r="297" spans="1:17">
       <c r="A297" t="s">
         <v>1</v>
       </c>
@@ -15862,7 +16180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298">
+    <row r="298" spans="1:17">
       <c r="A298" t="s">
         <v>1</v>
       </c>
@@ -15915,7 +16233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299">
+    <row r="299" spans="1:17">
       <c r="A299" t="s">
         <v>1</v>
       </c>
@@ -15968,7 +16286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300">
+    <row r="300" spans="1:17">
       <c r="A300" t="s">
         <v>1</v>
       </c>
@@ -16021,7 +16339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301">
+    <row r="301" spans="1:17">
       <c r="A301" t="s">
         <v>1</v>
       </c>
@@ -16074,7 +16392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302">
+    <row r="302" spans="1:17">
       <c r="A302" t="s">
         <v>1</v>
       </c>
@@ -16127,7 +16445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303">
+    <row r="303" spans="1:17">
       <c r="A303" t="s">
         <v>1</v>
       </c>
@@ -16180,7 +16498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304">
+    <row r="304" spans="1:17">
       <c r="A304" t="s">
         <v>1</v>
       </c>
@@ -16233,7 +16551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305">
+    <row r="305" spans="1:17">
       <c r="A305" t="s">
         <v>1</v>
       </c>
@@ -16286,7 +16604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306">
+    <row r="306" spans="1:17">
       <c r="A306" t="s">
         <v>1</v>
       </c>
@@ -16339,7 +16657,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307">
+    <row r="307" spans="1:17">
       <c r="A307" t="s">
         <v>1</v>
       </c>
@@ -16392,7 +16710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="308">
+    <row r="308" spans="1:17">
       <c r="A308" t="s">
         <v>1</v>
       </c>
@@ -16445,7 +16763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309">
+    <row r="309" spans="1:17">
       <c r="A309" t="s">
         <v>1</v>
       </c>
@@ -16498,7 +16816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="310">
+    <row r="310" spans="1:17">
       <c r="A310" t="s">
         <v>1</v>
       </c>
@@ -16551,7 +16869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311">
+    <row r="311" spans="1:17">
       <c r="A311" t="s">
         <v>1</v>
       </c>
@@ -16604,7 +16922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312">
+    <row r="312" spans="1:17">
       <c r="A312" t="s">
         <v>1</v>
       </c>
@@ -16657,7 +16975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313">
+    <row r="313" spans="1:17">
       <c r="A313" t="s">
         <v>1</v>
       </c>
@@ -16710,7 +17028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314">
+    <row r="314" spans="1:17">
       <c r="A314" t="s">
         <v>1</v>
       </c>
@@ -16763,7 +17081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315">
+    <row r="315" spans="1:17">
       <c r="A315" t="s">
         <v>1</v>
       </c>
@@ -16816,7 +17134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316">
+    <row r="316" spans="1:17">
       <c r="A316" t="s">
         <v>1</v>
       </c>
@@ -16869,7 +17187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317">
+    <row r="317" spans="1:17">
       <c r="A317" t="s">
         <v>1</v>
       </c>
@@ -16922,7 +17240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318">
+    <row r="318" spans="1:17">
       <c r="A318" t="s">
         <v>1</v>
       </c>
@@ -16975,7 +17293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319">
+    <row r="319" spans="1:17">
       <c r="A319" t="s">
         <v>1</v>
       </c>
@@ -17028,7 +17346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320">
+    <row r="320" spans="1:17">
       <c r="A320" t="s">
         <v>1</v>
       </c>
@@ -17081,7 +17399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321">
+    <row r="321" spans="1:17">
       <c r="A321" t="s">
         <v>1</v>
       </c>
@@ -17134,7 +17452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322">
+    <row r="322" spans="1:17">
       <c r="A322" t="s">
         <v>1</v>
       </c>
@@ -17187,7 +17505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323">
+    <row r="323" spans="1:17">
       <c r="A323" t="s">
         <v>1</v>
       </c>
@@ -17240,7 +17558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324">
+    <row r="324" spans="1:17">
       <c r="A324" t="s">
         <v>1</v>
       </c>
@@ -17293,7 +17611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325">
+    <row r="325" spans="1:17">
       <c r="A325" t="s">
         <v>1</v>
       </c>
@@ -17346,7 +17664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326">
+    <row r="326" spans="1:17">
       <c r="A326" t="s">
         <v>1</v>
       </c>
@@ -17399,7 +17717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="327">
+    <row r="327" spans="1:17">
       <c r="A327" t="s">
         <v>1</v>
       </c>
@@ -17452,7 +17770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="328">
+    <row r="328" spans="1:17">
       <c r="A328" t="s">
         <v>1</v>
       </c>
@@ -17505,7 +17823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="329">
+    <row r="329" spans="1:17">
       <c r="A329" t="s">
         <v>1</v>
       </c>
@@ -17558,7 +17876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330">
+    <row r="330" spans="1:17">
       <c r="A330" t="s">
         <v>1</v>
       </c>
@@ -17611,7 +17929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="331">
+    <row r="331" spans="1:17">
       <c r="A331" t="s">
         <v>1</v>
       </c>
@@ -17664,7 +17982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="332">
+    <row r="332" spans="1:17">
       <c r="A332" t="s">
         <v>1</v>
       </c>
@@ -17717,7 +18035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="333">
+    <row r="333" spans="1:17">
       <c r="A333" t="s">
         <v>1</v>
       </c>
@@ -17770,7 +18088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="334">
+    <row r="334" spans="1:17">
       <c r="A334" t="s">
         <v>1</v>
       </c>
@@ -17823,7 +18141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="335">
+    <row r="335" spans="1:17">
       <c r="A335" t="s">
         <v>1</v>
       </c>
@@ -17876,7 +18194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="336">
+    <row r="336" spans="1:17">
       <c r="A336" t="s">
         <v>1</v>
       </c>
@@ -17929,7 +18247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="337">
+    <row r="337" spans="1:17">
       <c r="A337" t="s">
         <v>1</v>
       </c>
@@ -17982,7 +18300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="338">
+    <row r="338" spans="1:17">
       <c r="A338" t="s">
         <v>1</v>
       </c>
@@ -18035,7 +18353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="339">
+    <row r="339" spans="1:17">
       <c r="A339" t="s">
         <v>1</v>
       </c>
@@ -18088,7 +18406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="340">
+    <row r="340" spans="1:17">
       <c r="A340" t="s">
         <v>1</v>
       </c>
@@ -18141,7 +18459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="341">
+    <row r="341" spans="1:17">
       <c r="A341" t="s">
         <v>1</v>
       </c>
@@ -18194,7 +18512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="342">
+    <row r="342" spans="1:17">
       <c r="A342" t="s">
         <v>1</v>
       </c>
@@ -18247,7 +18565,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="343">
+    <row r="343" spans="1:17">
       <c r="A343" t="s">
         <v>1</v>
       </c>
@@ -18300,7 +18618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="344">
+    <row r="344" spans="1:17">
       <c r="A344" t="s">
         <v>1</v>
       </c>
@@ -18353,7 +18671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="345">
+    <row r="345" spans="1:17">
       <c r="A345" t="s">
         <v>1</v>
       </c>
@@ -18406,7 +18724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="346">
+    <row r="346" spans="1:17">
       <c r="A346" t="s">
         <v>1</v>
       </c>
@@ -18459,7 +18777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="347">
+    <row r="347" spans="1:17">
       <c r="A347" t="s">
         <v>1</v>
       </c>
@@ -18512,7 +18830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="348">
+    <row r="348" spans="1:17">
       <c r="A348" t="s">
         <v>1</v>
       </c>
@@ -18565,7 +18883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="349">
+    <row r="349" spans="1:17">
       <c r="A349" t="s">
         <v>1</v>
       </c>
@@ -18618,7 +18936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="350">
+    <row r="350" spans="1:17">
       <c r="A350" t="s">
         <v>1</v>
       </c>
@@ -18671,7 +18989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="351">
+    <row r="351" spans="1:17">
       <c r="A351" t="s">
         <v>1</v>
       </c>
@@ -18724,7 +19042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="352">
+    <row r="352" spans="1:17">
       <c r="A352" t="s">
         <v>1</v>
       </c>
@@ -18777,7 +19095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="353">
+    <row r="353" spans="1:17">
       <c r="A353" t="s">
         <v>1</v>
       </c>
@@ -18830,7 +19148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="354">
+    <row r="354" spans="1:17">
       <c r="A354" t="s">
         <v>1</v>
       </c>
@@ -18883,7 +19201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="355">
+    <row r="355" spans="1:17">
       <c r="A355" t="s">
         <v>1</v>
       </c>
@@ -18936,7 +19254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="356">
+    <row r="356" spans="1:17">
       <c r="A356" t="s">
         <v>1</v>
       </c>
@@ -18989,7 +19307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="357">
+    <row r="357" spans="1:17">
       <c r="A357" t="s">
         <v>1</v>
       </c>
@@ -19042,7 +19360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="358">
+    <row r="358" spans="1:17">
       <c r="A358" t="s">
         <v>1</v>
       </c>
@@ -19095,7 +19413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="359">
+    <row r="359" spans="1:17">
       <c r="A359" t="s">
         <v>1</v>
       </c>
@@ -19148,7 +19466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="360">
+    <row r="360" spans="1:17">
       <c r="A360" t="s">
         <v>1</v>
       </c>
@@ -19201,7 +19519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="361">
+    <row r="361" spans="1:17">
       <c r="A361" t="s">
         <v>1</v>
       </c>
@@ -19254,7 +19572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="362">
+    <row r="362" spans="1:17">
       <c r="A362" t="s">
         <v>1</v>
       </c>
@@ -19307,7 +19625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="363">
+    <row r="363" spans="1:17">
       <c r="A363" t="s">
         <v>1</v>
       </c>
@@ -19360,7 +19678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="364">
+    <row r="364" spans="1:17">
       <c r="A364" t="s">
         <v>1</v>
       </c>
@@ -19413,7 +19731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="365">
+    <row r="365" spans="1:17">
       <c r="A365" t="s">
         <v>1</v>
       </c>
@@ -19466,7 +19784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="366">
+    <row r="366" spans="1:17">
       <c r="A366" t="s">
         <v>1</v>
       </c>
@@ -19519,7 +19837,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="367">
+    <row r="367" spans="1:17">
       <c r="A367" t="s">
         <v>1</v>
       </c>
@@ -19572,7 +19890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="368">
+    <row r="368" spans="1:17">
       <c r="A368" t="s">
         <v>1</v>
       </c>
@@ -19625,7 +19943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="369">
+    <row r="369" spans="1:17">
       <c r="A369" t="s">
         <v>1</v>
       </c>
@@ -19678,7 +19996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="370">
+    <row r="370" spans="1:17">
       <c r="A370" t="s">
         <v>1</v>
       </c>
@@ -19731,7 +20049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="371">
+    <row r="371" spans="1:17">
       <c r="A371" t="s">
         <v>1</v>
       </c>
@@ -19784,7 +20102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="372">
+    <row r="372" spans="1:17">
       <c r="A372" t="s">
         <v>1</v>
       </c>
@@ -19837,7 +20155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="373">
+    <row r="373" spans="1:17">
       <c r="A373" t="s">
         <v>1</v>
       </c>
@@ -19890,7 +20208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="374">
+    <row r="374" spans="1:17">
       <c r="A374" t="s">
         <v>1</v>
       </c>
@@ -19943,7 +20261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="375">
+    <row r="375" spans="1:17">
       <c r="A375" t="s">
         <v>1</v>
       </c>
@@ -19996,7 +20314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="376">
+    <row r="376" spans="1:17">
       <c r="A376" t="s">
         <v>1</v>
       </c>
@@ -20049,7 +20367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="377">
+    <row r="377" spans="1:17">
       <c r="A377" t="s">
         <v>1</v>
       </c>
@@ -20102,7 +20420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="378">
+    <row r="378" spans="1:17">
       <c r="A378" t="s">
         <v>1</v>
       </c>
@@ -20155,7 +20473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="379">
+    <row r="379" spans="1:17">
       <c r="A379" t="s">
         <v>1</v>
       </c>
@@ -20208,7 +20526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="380">
+    <row r="380" spans="1:17">
       <c r="A380" t="s">
         <v>1</v>
       </c>
@@ -20261,7 +20579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="381">
+    <row r="381" spans="1:17">
       <c r="A381" t="s">
         <v>1</v>
       </c>
@@ -20314,7 +20632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="382">
+    <row r="382" spans="1:17">
       <c r="A382" t="s">
         <v>1</v>
       </c>
@@ -20367,7 +20685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="383">
+    <row r="383" spans="1:17">
       <c r="A383" t="s">
         <v>1</v>
       </c>
@@ -20420,7 +20738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="384">
+    <row r="384" spans="1:17">
       <c r="A384" t="s">
         <v>1</v>
       </c>
@@ -20473,7 +20791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="385">
+    <row r="385" spans="1:17">
       <c r="A385" t="s">
         <v>1</v>
       </c>
@@ -20526,7 +20844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="386">
+    <row r="386" spans="1:17">
       <c r="A386" t="s">
         <v>1</v>
       </c>
@@ -20579,7 +20897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="387">
+    <row r="387" spans="1:17">
       <c r="A387" t="s">
         <v>1</v>
       </c>
@@ -20632,7 +20950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="388">
+    <row r="388" spans="1:17">
       <c r="A388" t="s">
         <v>1</v>
       </c>
@@ -20685,7 +21003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="389">
+    <row r="389" spans="1:17">
       <c r="A389" t="s">
         <v>1</v>
       </c>
@@ -20738,7 +21056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="390">
+    <row r="390" spans="1:17">
       <c r="A390" t="s">
         <v>1</v>
       </c>
@@ -20791,7 +21109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="391">
+    <row r="391" spans="1:17">
       <c r="A391" t="s">
         <v>1</v>
       </c>
@@ -20844,7 +21162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="392">
+    <row r="392" spans="1:17">
       <c r="A392" t="s">
         <v>1</v>
       </c>
@@ -20897,7 +21215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="393">
+    <row r="393" spans="1:17">
       <c r="A393" t="s">
         <v>1</v>
       </c>
@@ -20950,7 +21268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="394">
+    <row r="394" spans="1:17">
       <c r="A394" t="s">
         <v>1</v>
       </c>
@@ -21003,7 +21321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="395">
+    <row r="395" spans="1:17">
       <c r="A395" t="s">
         <v>1</v>
       </c>
@@ -21056,7 +21374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="396">
+    <row r="396" spans="1:17">
       <c r="A396" t="s">
         <v>1</v>
       </c>
@@ -21109,7 +21427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="397">
+    <row r="397" spans="1:17">
       <c r="A397" t="s">
         <v>1</v>
       </c>
@@ -21162,7 +21480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="398">
+    <row r="398" spans="1:17">
       <c r="A398" t="s">
         <v>1</v>
       </c>
@@ -21215,7 +21533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="399">
+    <row r="399" spans="1:17">
       <c r="A399" t="s">
         <v>1</v>
       </c>
@@ -21268,7 +21586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="400">
+    <row r="400" spans="1:17">
       <c r="A400" t="s">
         <v>1</v>
       </c>
@@ -21321,7 +21639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="401">
+    <row r="401" spans="1:17">
       <c r="A401" t="s">
         <v>1</v>
       </c>
@@ -21374,7 +21692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="402">
+    <row r="402" spans="1:17">
       <c r="A402" t="s">
         <v>1</v>
       </c>
@@ -21427,7 +21745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="403">
+    <row r="403" spans="1:17">
       <c r="A403" t="s">
         <v>1</v>
       </c>
@@ -21480,7 +21798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="404">
+    <row r="404" spans="1:17">
       <c r="A404" t="s">
         <v>1</v>
       </c>
@@ -21533,7 +21851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="405">
+    <row r="405" spans="1:17">
       <c r="A405" t="s">
         <v>1</v>
       </c>
@@ -21586,7 +21904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="406">
+    <row r="406" spans="1:17">
       <c r="A406" t="s">
         <v>1</v>
       </c>
@@ -21639,7 +21957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="407">
+    <row r="407" spans="1:17">
       <c r="A407" t="s">
         <v>1</v>
       </c>
@@ -21692,7 +22010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="408">
+    <row r="408" spans="1:17">
       <c r="A408" t="s">
         <v>1</v>
       </c>
@@ -21745,7 +22063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="409">
+    <row r="409" spans="1:17">
       <c r="A409" t="s">
         <v>1</v>
       </c>
@@ -21799,5 +22117,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>